<commit_message>
Update model outputs and sensitivity reporting to MAT-based scenario loading
</commit_message>
<xml_diff>
--- a/Code/dge-metric-model/ExcelFiles/ModelCalibration5Sectorsand1Regions.xlsx
+++ b/Code/dge-metric-model/ExcelFiles/ModelCalibration5Sectorsand1Regions.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAF904D-1057-4522-A625-5FE7C19C3310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="4" r:id="rId1"/>
@@ -123,7 +123,7 @@
     <definedName name="tauNH_p">Data!$AL$6</definedName>
     <definedName name="Y0_p">Data!$AL$3</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="649" uniqueCount="417">
   <si>
     <t>Sheets</t>
   </si>
@@ -1397,12 +1397,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1531,7 +1531,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1554,79 +1554,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFill="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="true"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="4"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="4" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="8" fillId="8" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="8" fillId="8" borderId="1" xfId="4" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="8" fillId="12" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="4" applyFont="true" applyFill="true"/>
+    <xf numFmtId="1" fontId="8" fillId="12" borderId="0" xfId="4" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="4" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="4" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFill="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Neutral 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Neutral 2" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1642,7 +1644,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1793,7 +1795,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1817,9 +1819,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1843,7 +1845,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1878,7 +1880,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1896,7 +1898,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1921,7 +1923,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -3683,17 +3685,17 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC00773-2217-4A15-8F36-7940A6632C72}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC00773-2217-4A15-8F36-7940A6632C72}">
   <dimension ref="A1:C158"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="true" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" style="4" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="122.5703125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="16" style="4" customWidth="true"/>
+    <col min="2" max="2" width="15.7109375" style="4" customWidth="true"/>
+    <col min="3" max="3" width="122.5703125" style="4" customWidth="true"/>
     <col min="4" max="16384" width="8.5703125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>48</v>
       </c>
@@ -3704,7 +3706,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>89</v>
       </c>
@@ -3715,7 +3717,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>328</v>
       </c>
@@ -3726,7 +3728,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>90</v>
       </c>
@@ -3737,7 +3739,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>329</v>
       </c>
@@ -3748,7 +3750,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>91</v>
       </c>
@@ -3759,7 +3761,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>92</v>
       </c>
@@ -3770,7 +3772,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>93</v>
       </c>
@@ -3781,7 +3783,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>94</v>
       </c>
@@ -3792,7 +3794,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>95</v>
       </c>
@@ -3803,7 +3805,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>412</v>
       </c>
@@ -3814,7 +3816,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>413</v>
       </c>
@@ -3825,7 +3827,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>414</v>
       </c>
@@ -3836,14 +3838,14 @@
         <v>227</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>96</v>
       </c>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
     </row>
-    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>97</v>
       </c>
@@ -3854,18 +3856,18 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>98</v>
       </c>
       <c r="B16" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>99</v>
       </c>
@@ -3876,7 +3878,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>100</v>
       </c>
@@ -3887,7 +3889,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>101</v>
       </c>
@@ -3898,14 +3900,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
         <v>102</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
     </row>
-    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>103</v>
       </c>
@@ -3916,7 +3918,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>104</v>
       </c>
@@ -3927,7 +3929,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>105</v>
       </c>
@@ -3938,7 +3940,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>106</v>
       </c>
@@ -3949,7 +3951,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>107</v>
       </c>
@@ -3960,14 +3962,14 @@
         <v>237</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
         <v>108</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
     </row>
-    <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>109</v>
       </c>
@@ -3978,7 +3980,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>110</v>
       </c>
@@ -3989,7 +3991,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>111</v>
       </c>
@@ -4000,7 +4002,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>112</v>
       </c>
@@ -4011,7 +4013,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>113</v>
       </c>
@@ -4022,14 +4024,14 @@
         <v>242</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
         <v>114</v>
       </c>
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
     </row>
-    <row r="33" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>115</v>
       </c>
@@ -4040,7 +4042,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>116</v>
       </c>
@@ -4051,7 +4053,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>117</v>
       </c>
@@ -4062,7 +4064,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>118</v>
       </c>
@@ -4073,7 +4075,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>119</v>
       </c>
@@ -4084,14 +4086,14 @@
         <v>247</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
         <v>120</v>
       </c>
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
     </row>
-    <row r="39" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>121</v>
       </c>
@@ -4102,7 +4104,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>122</v>
       </c>
@@ -4113,7 +4115,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>123</v>
       </c>
@@ -4124,7 +4126,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>124</v>
       </c>
@@ -4135,7 +4137,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>125</v>
       </c>
@@ -4146,14 +4148,14 @@
         <v>252</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A44" s="26" t="s">
         <v>330</v>
       </c>
       <c r="B44" s="27"/>
       <c r="C44" s="27"/>
     </row>
-    <row r="45" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>126</v>
       </c>
@@ -4164,7 +4166,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>127</v>
       </c>
@@ -4175,7 +4177,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>128</v>
       </c>
@@ -4186,7 +4188,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>129</v>
       </c>
@@ -4197,7 +4199,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>130</v>
       </c>
@@ -4208,14 +4210,14 @@
         <v>335</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A50" s="26" t="s">
         <v>336</v>
       </c>
       <c r="B50" s="27"/>
       <c r="C50" s="27"/>
     </row>
-    <row r="51" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>131</v>
       </c>
@@ -4226,7 +4228,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>132</v>
       </c>
@@ -4237,7 +4239,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>133</v>
       </c>
@@ -4248,7 +4250,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>134</v>
       </c>
@@ -4259,7 +4261,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>135</v>
       </c>
@@ -4270,14 +4272,14 @@
         <v>341</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A56" s="26">
         <v>1</v>
       </c>
       <c r="B56" s="27"/>
       <c r="C56" s="27"/>
     </row>
-    <row r="57" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="57" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>136</v>
       </c>
@@ -4288,7 +4290,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>137</v>
       </c>
@@ -4299,7 +4301,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="59" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>138</v>
       </c>
@@ -4310,7 +4312,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>139</v>
       </c>
@@ -4321,7 +4323,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="61" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>140</v>
       </c>
@@ -4332,14 +4334,14 @@
         <v>346</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="62" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A62" s="26" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="27"/>
       <c r="C62" s="27"/>
     </row>
-    <row r="63" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="63" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
         <v>142</v>
       </c>
@@ -4350,7 +4352,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="64" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>143</v>
       </c>
@@ -4361,7 +4363,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="65" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
         <v>144</v>
       </c>
@@ -4372,7 +4374,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="66" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>145</v>
       </c>
@@ -4383,7 +4385,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="67" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>146</v>
       </c>
@@ -4394,14 +4396,14 @@
         <v>257</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A68" s="26" t="s">
         <v>347</v>
       </c>
       <c r="B68" s="27"/>
       <c r="C68" s="27"/>
     </row>
-    <row r="69" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>147</v>
       </c>
@@ -4412,7 +4414,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="70" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>148</v>
       </c>
@@ -4423,7 +4425,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="71" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>149</v>
       </c>
@@ -4434,7 +4436,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="72" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>150</v>
       </c>
@@ -4445,7 +4447,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="73" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>151</v>
       </c>
@@ -4456,14 +4458,14 @@
         <v>352</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="74" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A74" s="26" t="s">
         <v>152</v>
       </c>
       <c r="B74" s="27"/>
       <c r="C74" s="27"/>
     </row>
-    <row r="75" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="75" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>153</v>
       </c>
@@ -4474,7 +4476,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="76" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>154</v>
       </c>
@@ -4485,7 +4487,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="77" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>155</v>
       </c>
@@ -4496,7 +4498,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="78" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>156</v>
       </c>
@@ -4507,7 +4509,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>157</v>
       </c>
@@ -4518,14 +4520,14 @@
         <v>262</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="80" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A80" s="26" t="s">
         <v>158</v>
       </c>
       <c r="B80" s="27"/>
       <c r="C80" s="27"/>
     </row>
-    <row r="81" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="81" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>159</v>
       </c>
@@ -4536,7 +4538,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="82" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>160</v>
       </c>
@@ -4547,7 +4549,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>161</v>
       </c>
@@ -4558,7 +4560,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>162</v>
       </c>
@@ -4569,7 +4571,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="85" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>163</v>
       </c>
@@ -4580,14 +4582,14 @@
         <v>267</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="86" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A86" s="26" t="s">
         <v>164</v>
       </c>
       <c r="B86" s="27"/>
       <c r="C86" s="27"/>
     </row>
-    <row r="87" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="87" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>165</v>
       </c>
@@ -4598,7 +4600,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="88" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>166</v>
       </c>
@@ -4609,7 +4611,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="89" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>167</v>
       </c>
@@ -4620,7 +4622,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="90" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>168</v>
       </c>
@@ -4631,7 +4633,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="91" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>169</v>
       </c>
@@ -4642,14 +4644,14 @@
         <v>272</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="92" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A92" s="26" t="s">
         <v>164</v>
       </c>
       <c r="B92" s="27"/>
       <c r="C92" s="27"/>
     </row>
-    <row r="93" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="93" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>353</v>
       </c>
@@ -4660,7 +4662,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="94" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>354</v>
       </c>
@@ -4671,7 +4673,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="95" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>355</v>
       </c>
@@ -4682,7 +4684,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="96" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
         <v>356</v>
       </c>
@@ -4693,7 +4695,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="97" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A97" s="4" t="s">
         <v>357</v>
       </c>
@@ -4704,14 +4706,14 @@
         <v>272</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="98" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A98" s="26" t="s">
         <v>170</v>
       </c>
       <c r="B98" s="27"/>
       <c r="C98" s="27"/>
     </row>
-    <row r="99" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="99" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
         <v>171</v>
       </c>
@@ -4722,7 +4724,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="100" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
         <v>172</v>
       </c>
@@ -4733,7 +4735,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="101" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>173</v>
       </c>
@@ -4744,7 +4746,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="102" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
         <v>174</v>
       </c>
@@ -4755,7 +4757,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="103" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>175</v>
       </c>
@@ -4766,7 +4768,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="104" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>176</v>
       </c>
@@ -4777,7 +4779,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="105" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>177</v>
       </c>
@@ -4788,7 +4790,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="106" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
         <v>178</v>
       </c>
@@ -4799,7 +4801,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="107" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>179</v>
       </c>
@@ -4810,7 +4812,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="108" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>180</v>
       </c>
@@ -4821,7 +4823,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="109" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>181</v>
       </c>
@@ -4832,7 +4834,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="110" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>182</v>
       </c>
@@ -4843,7 +4845,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="111" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>183</v>
       </c>
@@ -4854,7 +4856,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="112" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
         <v>184</v>
       </c>
@@ -4865,7 +4867,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="113" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
         <v>185</v>
       </c>
@@ -4876,7 +4878,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="114" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>186</v>
       </c>
@@ -4887,7 +4889,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="115" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>187</v>
       </c>
@@ -4898,7 +4900,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="116" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
         <v>188</v>
       </c>
@@ -4909,7 +4911,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="117" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
         <v>189</v>
       </c>
@@ -4920,7 +4922,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="118" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>190</v>
       </c>
@@ -4931,14 +4933,14 @@
         <v>292</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="119" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A119" s="26" t="s">
         <v>358</v>
       </c>
       <c r="B119" s="27"/>
       <c r="C119" s="27"/>
     </row>
-    <row r="120" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="120" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>191</v>
       </c>
@@ -4949,7 +4951,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="121" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
         <v>192</v>
       </c>
@@ -4960,7 +4962,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="122" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
         <v>193</v>
       </c>
@@ -4971,7 +4973,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="123" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
         <v>194</v>
       </c>
@@ -4982,7 +4984,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="124" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
         <v>195</v>
       </c>
@@ -4993,7 +4995,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="125" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
         <v>196</v>
       </c>
@@ -5004,7 +5006,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="126" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
         <v>197</v>
       </c>
@@ -5015,7 +5017,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="127" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
         <v>198</v>
       </c>
@@ -5026,7 +5028,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="128" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
         <v>199</v>
       </c>
@@ -5037,7 +5039,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="129" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
         <v>200</v>
       </c>
@@ -5048,7 +5050,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="130" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
         <v>201</v>
       </c>
@@ -5059,7 +5061,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="131" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
         <v>202</v>
       </c>
@@ -5070,7 +5072,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="132" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>203</v>
       </c>
@@ -5081,7 +5083,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="133" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
         <v>204</v>
       </c>
@@ -5092,7 +5094,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="134" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
         <v>205</v>
       </c>
@@ -5103,7 +5105,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="135" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
         <v>206</v>
       </c>
@@ -5114,7 +5116,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="136" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
         <v>207</v>
       </c>
@@ -5125,7 +5127,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="137" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
         <v>208</v>
       </c>
@@ -5136,7 +5138,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="138" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
         <v>209</v>
       </c>
@@ -5147,7 +5149,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="139" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
         <v>210</v>
       </c>
@@ -5158,14 +5160,14 @@
         <v>378</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="140" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A140" s="26" t="s">
         <v>211</v>
       </c>
       <c r="B140" s="27"/>
       <c r="C140" s="27"/>
     </row>
-    <row r="141" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="141" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
         <v>212</v>
       </c>
@@ -5176,7 +5178,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="142" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
         <v>213</v>
       </c>
@@ -5187,7 +5189,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="143" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
         <v>214</v>
       </c>
@@ -5198,7 +5200,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="144" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
         <v>215</v>
       </c>
@@ -5209,7 +5211,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="145" ht="14.45" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
         <v>216</v>
       </c>
@@ -5220,14 +5222,14 @@
         <v>297</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="146" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A146" s="26" t="s">
         <v>379</v>
       </c>
       <c r="B146" s="27"/>
       <c r="C146" s="27"/>
     </row>
-    <row r="147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="147" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
         <v>380</v>
       </c>
@@ -5238,7 +5240,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="148" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
         <v>382</v>
       </c>
@@ -5249,7 +5251,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="149" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
         <v>383</v>
       </c>
@@ -5260,7 +5262,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="150" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
         <v>384</v>
       </c>
@@ -5271,7 +5273,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="151" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
         <v>385</v>
       </c>
@@ -5282,14 +5284,14 @@
         <v>297</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="152" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A152" s="26" t="s">
         <v>386</v>
       </c>
       <c r="B152" s="27"/>
       <c r="C152" s="27"/>
     </row>
-    <row r="153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="153" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>387</v>
       </c>
@@ -5300,7 +5302,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="154" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
         <v>389</v>
       </c>
@@ -5311,7 +5313,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="155" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
         <v>391</v>
       </c>
@@ -5322,7 +5324,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="156" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
         <v>393</v>
       </c>
@@ -5333,7 +5335,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="157" ht="15" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
         <v>395</v>
       </c>
@@ -5344,7 +5346,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="158" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
         <v>415</v>
       </c>

</xml_diff>